<commit_message>
Changed status of all completed tasks (or those that will be by the time we submit)
</commit_message>
<xml_diff>
--- a/_reference/2026-05-02_BDA_Team-Pipeline_Ass01_ProjPlan.xlsx
+++ b/_reference/2026-05-02_BDA_Team-Pipeline_Ass01_ProjPlan.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Archive\BBK\BBK_03_MSc in Data Analytics\MSc_Y2_Big Data Analytics_BUCI065H7\S99_Assignments &amp; Exams\Assignments\40\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gmmur\Documents\Big Data Analytics\bda-proj\BDA-teamwork\_reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="234" documentId="13_ncr:1_{B188FCD7-1158-414F-88EA-588F343108C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1C4A06F1-5B2B-4E34-B117-386209BE8CA7}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A0F0885-2C6B-455D-BC78-8A8F882EF71F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -306,6 +306,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">Initialize GitHub Repo &amp; </t>
@@ -316,6 +317,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>invite steliosot</t>
@@ -483,6 +485,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">Record a screen-share demo and have each member explain their contribution (per Section 10).
@@ -495,6 +498,7 @@
         <sz val="11"/>
         <color rgb="FFFF0000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>(***NOTE: THE INDIVIDUAL ASSIGNMENT IS MADE AVAILABLE THIS WEEK***)</t>
@@ -510,6 +514,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">NOTE: Mon, 25-May-2026 is a Bank Holiday
@@ -520,6 +525,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>Compile edit. Add captions, etc.</t>
@@ -877,6 +883,7 @@
         <sz val="12"/>
         <color rgb="FFFF0000"/>
         <rFont val="Segoe UI"/>
+        <family val="2"/>
       </rPr>
       <t>Gemini API</t>
     </r>
@@ -885,6 +892,7 @@
         <sz val="12"/>
         <color rgb="FF1F2328"/>
         <rFont val="Segoe UI"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> for transcript correction</t>
     </r>
@@ -1118,7 +1126,7 @@
     <numFmt numFmtId="164" formatCode="yyyy/mm/dd;@"/>
     <numFmt numFmtId="165" formatCode="ddd\,\ dd\-mmm\-yyyy"/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="25" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1130,6 +1138,7 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1256,12 +1265,14 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1293,19 +1304,13 @@
       <sz val="12"/>
       <color rgb="FFFF0000"/>
       <name val="Segoe UI"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
       <color rgb="FF1F2328"/>
       <name val="Segoe UI"/>
-    </font>
-    <font>
-      <b/>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="7">
@@ -1551,18 +1556,146 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="5" xfId="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="5" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="92">
+  <dxfs count="70">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1707,6 +1840,12 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -1744,339 +1883,6 @@
     </dxf>
     <dxf>
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -2196,14 +2002,14 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{9D73516B-3E52-443E-B205-B6EE6F647340}" name="Table8" displayName="Table8" ref="A15:E18" totalsRowShown="0" dataDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{9D73516B-3E52-443E-B205-B6EE6F647340}" name="Table8" displayName="Table8" ref="A15:E18" totalsRowShown="0" dataDxfId="25">
   <autoFilter ref="A15:E18" xr:uid="{9D73516B-3E52-443E-B205-B6EE6F647340}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{E60A5273-5C84-453D-8EC1-C6541773BC60}" name="timestamp" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{BC1CE138-C891-45C3-95AB-E9D78A4F4CE2}" name="name" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{FE0D840B-9360-406D-9DEC-A856F7DB8652}" name="raw_text_vosk" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{7EEB9BAF-3AFE-4568-94B3-303617527D23}" name="text" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{98F79F26-2A41-492F-B308-CF63480B055F}" name="time_taken_sec" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{E60A5273-5C84-453D-8EC1-C6541773BC60}" name="timestamp" dataDxfId="24"/>
+    <tableColumn id="2" xr3:uid="{BC1CE138-C891-45C3-95AB-E9D78A4F4CE2}" name="name" dataDxfId="23"/>
+    <tableColumn id="3" xr3:uid="{FE0D840B-9360-406D-9DEC-A856F7DB8652}" name="raw_text_vosk" dataDxfId="22"/>
+    <tableColumn id="4" xr3:uid="{7EEB9BAF-3AFE-4568-94B3-303617527D23}" name="text" dataDxfId="21"/>
+    <tableColumn id="5" xr3:uid="{98F79F26-2A41-492F-B308-CF63480B055F}" name="time_taken_sec" dataDxfId="20"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2216,12 +2022,12 @@
     <tableColumn id="1" xr3:uid="{EAB16663-796A-4D80-B59A-ECBB4CE8EE81}" name="timestamp"/>
     <tableColumn id="2" xr3:uid="{6E2785DC-02D0-4645-9F83-6BD2B353DC1E}" name="name"/>
     <tableColumn id="3" xr3:uid="{7EF23D8F-2EA6-47A8-8CA5-ED15CFBB9F4B}" name="text"/>
-    <tableColumn id="4" xr3:uid="{7872B727-A3E9-4175-9DC0-E78C9CB790B4}" name="time_taken_sec" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{AD123B6F-D646-442F-BAF2-3D4934D07E75}" name="question_flag" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{19406CDC-7D9B-4EF7-9658-7B207E673287}" name="num_words" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{F10E2254-038C-48F6-B11B-C49875D22ABE}" name="text_size_chars" dataDxfId="2"/>
-    <tableColumn id="8" xr3:uid="{9529BA64-4165-4908-BC51-B83A06A198F9}" name="speech_rate_wps" dataDxfId="1"/>
-    <tableColumn id="9" xr3:uid="{C353E353-9E68-4106-B418-0E65F70D1F6F}" name="speaker_turn_id" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{7872B727-A3E9-4175-9DC0-E78C9CB790B4}" name="time_taken_sec" dataDxfId="19"/>
+    <tableColumn id="5" xr3:uid="{AD123B6F-D646-442F-BAF2-3D4934D07E75}" name="question_flag" dataDxfId="18"/>
+    <tableColumn id="6" xr3:uid="{19406CDC-7D9B-4EF7-9658-7B207E673287}" name="num_words" dataDxfId="17"/>
+    <tableColumn id="7" xr3:uid="{F10E2254-038C-48F6-B11B-C49875D22ABE}" name="text_size_chars" dataDxfId="16"/>
+    <tableColumn id="8" xr3:uid="{9529BA64-4165-4908-BC51-B83A06A198F9}" name="speech_rate_wps" dataDxfId="15"/>
+    <tableColumn id="9" xr3:uid="{C353E353-9E68-4106-B418-0E65F70D1F6F}" name="speaker_turn_id" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2242,7 +2048,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{84BAE923-46F1-4CA5-A2DD-1F7E9839F945}" name="Table11" displayName="Table11" ref="G1:O24" totalsRowShown="0">
   <autoFilter ref="G1:O24" xr:uid="{84BAE923-46F1-4CA5-A2DD-1F7E9839F945}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{701E7413-613D-4A19-8134-14906B715480}" name="Proposed Team Name" dataDxfId="62"/>
+    <tableColumn id="1" xr3:uid="{701E7413-613D-4A19-8134-14906B715480}" name="Proposed Team Name" dataDxfId="57"/>
     <tableColumn id="2" xr3:uid="{8061771C-5AA5-43F6-BBD6-931BE60B943D}" name="Proposed by"/>
     <tableColumn id="3" xr3:uid="{D289F9B0-4897-41D4-B2D4-5A29DEEE758D}" name="Carys"/>
     <tableColumn id="4" xr3:uid="{B015474C-6BCE-4DAE-9235-E010C07C1DF7}" name="Gary"/>
@@ -2250,7 +2056,7 @@
     <tableColumn id="6" xr3:uid="{E3032E10-8CA9-4C46-A1A6-A4013F3C9226}" name="Mei Len"/>
     <tableColumn id="7" xr3:uid="{52424370-E8C7-47DF-9723-9EC1231EB24C}" name="Samuel"/>
     <tableColumn id="8" xr3:uid="{406083C9-9B78-423C-A1A2-30F2651CE2F1}" name="Toby"/>
-    <tableColumn id="9" xr3:uid="{013D8C47-04D7-4DBF-9623-4C4B462EA740}" name="Vote Count" dataDxfId="61">
+    <tableColumn id="9" xr3:uid="{013D8C47-04D7-4DBF-9623-4C4B462EA740}" name="Vote Count" dataDxfId="56">
       <calculatedColumnFormula>COUNTA(Table11[[#This Row],[Carys]:[Toby]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2259,33 +2065,33 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{3D05EDC5-ACB3-4ADA-8507-44E361F31599}" name="Table3" displayName="Table3" ref="A1:J19" totalsRowShown="0" headerRowDxfId="53" dataDxfId="52">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{3D05EDC5-ACB3-4ADA-8507-44E361F31599}" name="Table3" displayName="Table3" ref="A1:J19" totalsRowShown="0" headerRowDxfId="69" dataDxfId="68">
   <autoFilter ref="A1:J19" xr:uid="{3D05EDC5-ACB3-4ADA-8507-44E361F31599}"/>
   <tableColumns count="10">
-    <tableColumn id="10" xr3:uid="{8B7556E2-4DA3-4929-91F3-0B3DDC40C06B}" name="Sequence No." dataDxfId="51"/>
-    <tableColumn id="1" xr3:uid="{D98C609B-E0BE-4FDD-B5C2-EC3C9A082E2F}" name="Phase" dataDxfId="50"/>
-    <tableColumn id="2" xr3:uid="{E20FA66A-501E-4835-B5C3-78BC55BDE8C1}" name="Task" dataDxfId="49"/>
-    <tableColumn id="3" xr3:uid="{53A4E16C-749D-4649-8CEF-B05A04F89683}" name="Assignee" dataDxfId="48"/>
-    <tableColumn id="4" xr3:uid="{D9A5F161-F2B3-4604-B9B4-CEAA01441E7E}" name="Start Date" dataDxfId="47"/>
-    <tableColumn id="5" xr3:uid="{97B08F6E-A853-4861-991B-602712A3B541}" name="End Date" dataDxfId="46"/>
-    <tableColumn id="9" xr3:uid="{FA248AD3-C33A-45C3-B8ED-4ED870AB7537}" name="Days Count" dataDxfId="45">
+    <tableColumn id="10" xr3:uid="{8B7556E2-4DA3-4929-91F3-0B3DDC40C06B}" name="Sequence No." dataDxfId="67"/>
+    <tableColumn id="1" xr3:uid="{D98C609B-E0BE-4FDD-B5C2-EC3C9A082E2F}" name="Phase" dataDxfId="66"/>
+    <tableColumn id="2" xr3:uid="{E20FA66A-501E-4835-B5C3-78BC55BDE8C1}" name="Task" dataDxfId="65"/>
+    <tableColumn id="3" xr3:uid="{53A4E16C-749D-4649-8CEF-B05A04F89683}" name="Assignee" dataDxfId="64"/>
+    <tableColumn id="4" xr3:uid="{D9A5F161-F2B3-4604-B9B4-CEAA01441E7E}" name="Start Date" dataDxfId="63"/>
+    <tableColumn id="5" xr3:uid="{97B08F6E-A853-4861-991B-602712A3B541}" name="End Date" dataDxfId="62"/>
+    <tableColumn id="9" xr3:uid="{FA248AD3-C33A-45C3-B8ED-4ED870AB7537}" name="Days Count" dataDxfId="61">
       <calculatedColumnFormula>Table3[[#This Row],[End Date]]-Table3[[#This Row],[Start Date]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{9F2F7A0C-7D19-4DF0-9DA2-3DE3EB44E17F}" name="Status" dataDxfId="44"/>
-    <tableColumn id="7" xr3:uid="{75D03508-25A3-4482-A564-EBECC4052AE4}" name="Deliverable" dataDxfId="43"/>
-    <tableColumn id="8" xr3:uid="{019D1DB2-B63F-4461-83C6-4B023A33D72F}" name="Notes" dataDxfId="42"/>
+    <tableColumn id="6" xr3:uid="{9F2F7A0C-7D19-4DF0-9DA2-3DE3EB44E17F}" name="Status" dataDxfId="60"/>
+    <tableColumn id="7" xr3:uid="{75D03508-25A3-4482-A564-EBECC4052AE4}" name="Deliverable" dataDxfId="59"/>
+    <tableColumn id="8" xr3:uid="{019D1DB2-B63F-4461-83C6-4B023A33D72F}" name="Notes" dataDxfId="58"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{79369338-09EE-4B30-B5F1-EBB5519FB1CF}" name="Table1" displayName="Table1" ref="A7:C13" totalsRowShown="0" headerRowDxfId="41" dataDxfId="40">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{79369338-09EE-4B30-B5F1-EBB5519FB1CF}" name="Table1" displayName="Table1" ref="A7:C13" totalsRowShown="0" headerRowDxfId="55" dataDxfId="54">
   <autoFilter ref="A7:C13" xr:uid="{79369338-09EE-4B30-B5F1-EBB5519FB1CF}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{3B6E8B81-2F84-4D7E-918A-9D88F8502CD9}" name="Role" dataDxfId="39"/>
-    <tableColumn id="2" xr3:uid="{47656457-6CF2-4BD5-B749-AA52333B1AFC}" name="Team_Member_No" dataDxfId="38"/>
-    <tableColumn id="3" xr3:uid="{F993563A-5FFD-4B2F-AC69-11527B498F26}" name="Team_Member_Name" dataDxfId="37"/>
+    <tableColumn id="1" xr3:uid="{3B6E8B81-2F84-4D7E-918A-9D88F8502CD9}" name="Role" dataDxfId="53"/>
+    <tableColumn id="2" xr3:uid="{47656457-6CF2-4BD5-B749-AA52333B1AFC}" name="Team_Member_No" dataDxfId="52"/>
+    <tableColumn id="3" xr3:uid="{F993563A-5FFD-4B2F-AC69-11527B498F26}" name="Team_Member_Name" dataDxfId="51"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2295,55 +2101,55 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{3B51CB57-6C2F-4152-BA00-E49BFD7BEC62}" name="Table2" displayName="Table2" ref="A1:C4" totalsRowShown="0">
   <autoFilter ref="A1:C4" xr:uid="{3B51CB57-6C2F-4152-BA00-E49BFD7BEC62}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{C31B9A1A-8EB0-4617-8460-F8EBDDC5F974}" name="Role" dataDxfId="36"/>
-    <tableColumn id="2" xr3:uid="{86D9459E-A4B7-4180-860D-B66BF8585F61}" name="Team_Member_Pair" dataDxfId="35"/>
-    <tableColumn id="3" xr3:uid="{6BFEFD5F-3B6D-4D1F-A668-5EAA974FF596}" name="Task" dataDxfId="34"/>
+    <tableColumn id="1" xr3:uid="{C31B9A1A-8EB0-4617-8460-F8EBDDC5F974}" name="Role" dataDxfId="50"/>
+    <tableColumn id="2" xr3:uid="{86D9459E-A4B7-4180-860D-B66BF8585F61}" name="Team_Member_Pair" dataDxfId="49"/>
+    <tableColumn id="3" xr3:uid="{6BFEFD5F-3B6D-4D1F-A668-5EAA974FF596}" name="Task" dataDxfId="48"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{3DED07B8-3B29-4CE6-8D7D-81D302F66365}" name="Table_Script_Sequential" displayName="Table_Script_Sequential" ref="A5:D36" totalsRowShown="0" headerRowDxfId="33" dataDxfId="32">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{3DED07B8-3B29-4CE6-8D7D-81D302F66365}" name="Table_Script_Sequential" displayName="Table_Script_Sequential" ref="A5:D36" totalsRowShown="0" headerRowDxfId="47" dataDxfId="46">
   <autoFilter ref="A5:D36" xr:uid="{3DED07B8-3B29-4CE6-8D7D-81D302F66365}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{441B0C42-ECF5-4AA8-AC5B-8CF2435CB8DC}" name="Turn Count" dataDxfId="31"/>
-    <tableColumn id="2" xr3:uid="{3C989E8D-3824-4029-BA91-C5D26338B6B7}" name="Speaker_Number" dataDxfId="30"/>
-    <tableColumn id="4" xr3:uid="{107DEE54-DAB3-4382-A74C-F32991E35098}" name="Team_Member_Name" dataDxfId="29"/>
-    <tableColumn id="3" xr3:uid="{A4178B81-73F4-4F4A-8DCB-15617DA04B27}" name="Speech" dataDxfId="28"/>
+    <tableColumn id="1" xr3:uid="{441B0C42-ECF5-4AA8-AC5B-8CF2435CB8DC}" name="Turn Count" dataDxfId="45"/>
+    <tableColumn id="2" xr3:uid="{3C989E8D-3824-4029-BA91-C5D26338B6B7}" name="Speaker_Number" dataDxfId="44"/>
+    <tableColumn id="4" xr3:uid="{107DEE54-DAB3-4382-A74C-F32991E35098}" name="Team_Member_Name" dataDxfId="43"/>
+    <tableColumn id="3" xr3:uid="{A4178B81-73F4-4F4A-8DCB-15617DA04B27}" name="Speech" dataDxfId="42"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{A7F55938-32F3-4AA9-8652-9A9138AA6429}" name="Table_Script_NonSequential" displayName="Table_Script_NonSequential" ref="G5:J36" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{A7F55938-32F3-4AA9-8652-9A9138AA6429}" name="Table_Script_NonSequential" displayName="Table_Script_NonSequential" ref="G5:J36" totalsRowShown="0" headerRowDxfId="41" dataDxfId="40">
   <autoFilter ref="G5:J36" xr:uid="{A7F55938-32F3-4AA9-8652-9A9138AA6429}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="G6:J35">
     <sortCondition ref="G5:G35"/>
   </sortState>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{DD8D006E-7190-42A7-AB66-5E125A42F27F}" name="Turn Count" dataDxfId="25"/>
-    <tableColumn id="2" xr3:uid="{3E3C6106-E299-49D9-A753-0FF4B0FBF337}" name="Speaker_Number" dataDxfId="24"/>
-    <tableColumn id="3" xr3:uid="{98EADBE7-D226-4D87-BCFB-457243F29244}" name="Team_Member_Name" dataDxfId="23"/>
-    <tableColumn id="4" xr3:uid="{A93826DA-55E1-429D-873D-71E875C621A2}" name="Speech" dataDxfId="22"/>
+    <tableColumn id="1" xr3:uid="{DD8D006E-7190-42A7-AB66-5E125A42F27F}" name="Turn Count" dataDxfId="39"/>
+    <tableColumn id="2" xr3:uid="{3E3C6106-E299-49D9-A753-0FF4B0FBF337}" name="Speaker_Number" dataDxfId="38"/>
+    <tableColumn id="3" xr3:uid="{98EADBE7-D226-4D87-BCFB-457243F29244}" name="Team_Member_Name" dataDxfId="37"/>
+    <tableColumn id="4" xr3:uid="{A93826DA-55E1-429D-873D-71E875C621A2}" name="Speech" dataDxfId="36"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{E35BF121-281B-45CE-9A1E-748323E7CE52}" name="Table4" displayName="Table4" ref="A1:H11" totalsRowShown="0" headerRowDxfId="21" dataDxfId="20">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{E35BF121-281B-45CE-9A1E-748323E7CE52}" name="Table4" displayName="Table4" ref="A1:H11" totalsRowShown="0" headerRowDxfId="35" dataDxfId="34">
   <autoFilter ref="A1:H11" xr:uid="{E35BF121-281B-45CE-9A1E-748323E7CE52}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{748E1F5B-8FBF-4193-A340-8E5C2D9B4255}" name="Column Name" dataDxfId="19"/>
-    <tableColumn id="2" xr3:uid="{2DC0527E-F527-49CE-818E-84715CB496CB}" name="Source" dataDxfId="18"/>
-    <tableColumn id="3" xr3:uid="{D523D9CB-29AE-4C6E-ABC2-E8FF85E59DE3}" name="Type" dataDxfId="17"/>
-    <tableColumn id="4" xr3:uid="{F1BBA85D-DC41-4464-A469-EB6C804D1061}" name="Description/Logic" dataDxfId="16"/>
-    <tableColumn id="9" xr3:uid="{F0D57AEC-29BB-4869-BE86-4AFF923E0978}" name="Task Start" dataDxfId="15"/>
-    <tableColumn id="10" xr3:uid="{D09FD650-59F2-4F48-A30D-057C5D51042E}" name="Task End" dataDxfId="14"/>
-    <tableColumn id="5" xr3:uid="{29D8647A-34A5-4258-9B25-7A65C92D7808}" name="Role" dataDxfId="13"/>
-    <tableColumn id="7" xr3:uid="{ED84A4AA-F933-424F-A06B-33DA14667523}" name="Name " dataDxfId="12"/>
+    <tableColumn id="1" xr3:uid="{748E1F5B-8FBF-4193-A340-8E5C2D9B4255}" name="Column Name" dataDxfId="33"/>
+    <tableColumn id="2" xr3:uid="{2DC0527E-F527-49CE-818E-84715CB496CB}" name="Source" dataDxfId="32"/>
+    <tableColumn id="3" xr3:uid="{D523D9CB-29AE-4C6E-ABC2-E8FF85E59DE3}" name="Type" dataDxfId="31"/>
+    <tableColumn id="4" xr3:uid="{F1BBA85D-DC41-4464-A469-EB6C804D1061}" name="Description/Logic" dataDxfId="30"/>
+    <tableColumn id="9" xr3:uid="{F0D57AEC-29BB-4869-BE86-4AFF923E0978}" name="Task Start" dataDxfId="29"/>
+    <tableColumn id="10" xr3:uid="{D09FD650-59F2-4F48-A30D-057C5D51042E}" name="Task End" dataDxfId="28"/>
+    <tableColumn id="5" xr3:uid="{29D8647A-34A5-4258-9B25-7A65C92D7808}" name="Role" dataDxfId="27"/>
+    <tableColumn id="7" xr3:uid="{ED84A4AA-F933-424F-A06B-33DA14667523}" name="Name " dataDxfId="26"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2635,7 +2441,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B1BFCEB-859E-45C1-9561-8210E54A32F4}">
   <dimension ref="A1:O24"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="29.140625" bestFit="1" customWidth="1"/>
@@ -2654,7 +2460,7 @@
     <col min="15" max="15" width="13.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2695,7 +2501,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:15">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -2719,7 +2525,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:15">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>18</v>
       </c>
@@ -2743,7 +2549,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:15">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>23</v>
       </c>
@@ -2767,7 +2573,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:15">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>28</v>
       </c>
@@ -2791,7 +2597,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:15">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>33</v>
       </c>
@@ -2815,7 +2621,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:15">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>38</v>
       </c>
@@ -2839,7 +2645,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:15">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="D8" s="3" t="s">
         <v>43</v>
       </c>
@@ -2857,7 +2663,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:15">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>46</v>
       </c>
@@ -2875,7 +2681,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:15">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="42" t="s">
         <v>0</v>
       </c>
@@ -2909,7 +2715,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:15">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="43" t="s">
         <v>13</v>
       </c>
@@ -2930,7 +2736,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:15">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="44" t="s">
         <v>18</v>
       </c>
@@ -2948,7 +2754,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:15" ht="30.75">
+    <row r="13" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="43" t="s">
         <v>23</v>
       </c>
@@ -2966,7 +2772,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:15" ht="45.75">
+    <row r="14" spans="1:15" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="44" t="s">
         <v>28</v>
       </c>
@@ -2981,7 +2787,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:15" ht="30.75">
+    <row r="15" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="43" t="s">
         <v>33</v>
       </c>
@@ -2999,7 +2805,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:15" ht="45.75">
+    <row r="16" spans="1:15" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" s="45" t="s">
         <v>38</v>
       </c>
@@ -3017,7 +2823,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="7:15">
+    <row r="17" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G17" s="24" t="s">
         <v>60</v>
       </c>
@@ -3026,7 +2832,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="7:15">
+    <row r="18" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G18" s="24" t="s">
         <v>60</v>
       </c>
@@ -3035,7 +2841,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="7:15">
+    <row r="19" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G19" s="24" t="s">
         <v>60</v>
       </c>
@@ -3044,7 +2850,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="7:15">
+    <row r="20" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G20" s="24" t="s">
         <v>60</v>
       </c>
@@ -3053,7 +2859,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="7:15">
+    <row r="21" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G21" s="24" t="s">
         <v>60</v>
       </c>
@@ -3062,7 +2868,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="7:15">
+    <row r="22" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G22" s="24" t="s">
         <v>60</v>
       </c>
@@ -3071,7 +2877,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="7:15">
+    <row r="23" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G23" s="24" t="s">
         <v>60</v>
       </c>
@@ -3080,7 +2886,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="7:15">
+    <row r="24" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G24" s="24" t="s">
         <v>60</v>
       </c>
@@ -3090,101 +2896,29 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="D2">
-    <cfRule type="containsText" dxfId="91" priority="29" operator="containsText" text="Backlog">
+  <conditionalFormatting sqref="D2:D8">
+    <cfRule type="containsText" dxfId="13" priority="7" operator="containsText" text="Backlog">
       <formula>NOT(ISERROR(SEARCH("Backlog",D2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D3">
-    <cfRule type="containsText" dxfId="90" priority="22" operator="containsText" text="Overdue">
+  <conditionalFormatting sqref="D3:D8">
+    <cfRule type="containsText" dxfId="12" priority="1" operator="containsText" text="Overdue">
       <formula>NOT(ISERROR(SEARCH("Overdue",D3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="89" priority="23" operator="containsText" text="Blocked">
+    <cfRule type="containsText" dxfId="11" priority="2" operator="containsText" text="Blocked">
       <formula>NOT(ISERROR(SEARCH("Blocked",D3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="88" priority="24" operator="containsText" text="Cancelled">
+    <cfRule type="containsText" dxfId="10" priority="3" operator="containsText" text="Cancelled">
       <formula>NOT(ISERROR(SEARCH("Cancelled",D3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="87" priority="25" operator="containsText" text="Completed">
+    <cfRule type="containsText" dxfId="9" priority="4" operator="containsText" text="Completed">
       <formula>NOT(ISERROR(SEARCH("Completed",D3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="86" priority="26" operator="containsText" text="In Progress">
+    <cfRule type="containsText" dxfId="8" priority="5" operator="containsText" text="In Progress">
       <formula>NOT(ISERROR(SEARCH("In Progress",D3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="85" priority="27" operator="containsText" text="Planned">
+    <cfRule type="containsText" dxfId="7" priority="6" operator="containsText" text="Planned">
       <formula>NOT(ISERROR(SEARCH("Planned",D3)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="84" priority="28" operator="containsText" text="Backlog">
-      <formula>NOT(ISERROR(SEARCH("Backlog",D3)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D4">
-    <cfRule type="containsText" dxfId="83" priority="15" operator="containsText" text="Overdue">
-      <formula>NOT(ISERROR(SEARCH("Overdue",D4)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="82" priority="16" operator="containsText" text="Blocked">
-      <formula>NOT(ISERROR(SEARCH("Blocked",D4)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="81" priority="17" operator="containsText" text="Cancelled">
-      <formula>NOT(ISERROR(SEARCH("Cancelled",D4)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="80" priority="18" operator="containsText" text="Completed">
-      <formula>NOT(ISERROR(SEARCH("Completed",D4)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="79" priority="19" operator="containsText" text="In Progress">
-      <formula>NOT(ISERROR(SEARCH("In Progress",D4)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="78" priority="20" operator="containsText" text="Planned">
-      <formula>NOT(ISERROR(SEARCH("Planned",D4)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="77" priority="21" operator="containsText" text="Backlog">
-      <formula>NOT(ISERROR(SEARCH("Backlog",D4)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D5">
-    <cfRule type="containsText" dxfId="76" priority="8" operator="containsText" text="Overdue">
-      <formula>NOT(ISERROR(SEARCH("Overdue",D5)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="75" priority="9" operator="containsText" text="Blocked">
-      <formula>NOT(ISERROR(SEARCH("Blocked",D5)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="74" priority="10" operator="containsText" text="Cancelled">
-      <formula>NOT(ISERROR(SEARCH("Cancelled",D5)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="73" priority="11" operator="containsText" text="Completed">
-      <formula>NOT(ISERROR(SEARCH("Completed",D5)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="72" priority="12" operator="containsText" text="In Progress">
-      <formula>NOT(ISERROR(SEARCH("In Progress",D5)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="71" priority="13" operator="containsText" text="Planned">
-      <formula>NOT(ISERROR(SEARCH("Planned",D5)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="70" priority="14" operator="containsText" text="Backlog">
-      <formula>NOT(ISERROR(SEARCH("Backlog",D5)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D6:D8">
-    <cfRule type="containsText" dxfId="69" priority="1" operator="containsText" text="Overdue">
-      <formula>NOT(ISERROR(SEARCH("Overdue",D6)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="68" priority="2" operator="containsText" text="Blocked">
-      <formula>NOT(ISERROR(SEARCH("Blocked",D6)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="67" priority="3" operator="containsText" text="Cancelled">
-      <formula>NOT(ISERROR(SEARCH("Cancelled",D6)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="66" priority="4" operator="containsText" text="Completed">
-      <formula>NOT(ISERROR(SEARCH("Completed",D6)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="65" priority="5" operator="containsText" text="In Progress">
-      <formula>NOT(ISERROR(SEARCH("In Progress",D6)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="64" priority="6" operator="containsText" text="Planned">
-      <formula>NOT(ISERROR(SEARCH("Planned",D6)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="63" priority="7" operator="containsText" text="Backlog">
-      <formula>NOT(ISERROR(SEARCH("Backlog",D6)))</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
@@ -3206,7 +2940,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J22"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.140625" customWidth="1"/>
     <col min="2" max="2" width="15.7109375" bestFit="1" customWidth="1"/>
@@ -3221,7 +2955,7 @@
     <col min="11" max="11" width="5.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="30">
+    <row r="1" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>61</v>
       </c>
@@ -3253,7 +2987,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="45.75">
+    <row r="2" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="32">
         <v>1</v>
       </c>
@@ -3286,7 +3020,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="30.75">
+    <row r="3" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="11">
         <v>2</v>
       </c>
@@ -3319,7 +3053,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="45.75">
+    <row r="4" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="11">
         <v>3</v>
       </c>
@@ -3352,7 +3086,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="60.75">
+    <row r="5" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" s="11">
         <v>4</v>
       </c>
@@ -3385,7 +3119,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="76.5">
+    <row r="6" spans="1:10" ht="75" x14ac:dyDescent="0.25">
       <c r="A6" s="31">
         <v>5</v>
       </c>
@@ -3418,7 +3152,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="30.75">
+    <row r="7" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="11">
         <v>6</v>
       </c>
@@ -3451,7 +3185,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="30.75">
+    <row r="8" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="11">
         <v>7</v>
       </c>
@@ -3484,7 +3218,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="106.5">
+    <row r="9" spans="1:10" ht="105" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
         <v>8</v>
       </c>
@@ -3517,7 +3251,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="60.75">
+    <row r="10" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A10" s="31">
         <v>9</v>
       </c>
@@ -3550,7 +3284,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="30.75">
+    <row r="11" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
         <v>10</v>
       </c>
@@ -3583,7 +3317,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="30.75">
+    <row r="12" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="11">
         <v>11</v>
       </c>
@@ -3616,7 +3350,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="30.75">
+    <row r="13" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
         <v>12</v>
       </c>
@@ -3649,7 +3383,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="76.5">
+    <row r="14" spans="1:10" ht="75" x14ac:dyDescent="0.25">
       <c r="A14" s="11">
         <v>13</v>
       </c>
@@ -3678,11 +3412,11 @@
       <c r="I14" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="J14" s="51" t="s">
+      <c r="J14" s="50" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="30.75">
+    <row r="15" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="11">
         <v>14</v>
       </c>
@@ -3706,7 +3440,7 @@
         <v>5</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="I15" s="3" t="s">
         <v>115</v>
@@ -3715,7 +3449,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="76.5">
+    <row r="16" spans="1:10" ht="75" x14ac:dyDescent="0.25">
       <c r="A16" s="30">
         <v>15</v>
       </c>
@@ -3739,7 +3473,7 @@
         <v>1</v>
       </c>
       <c r="H16" s="23" t="s">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="I16" s="23" t="s">
         <v>73</v>
@@ -3748,7 +3482,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="45.75">
+    <row r="17" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A17" s="11">
         <v>16</v>
       </c>
@@ -3772,7 +3506,7 @@
         <v>1</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="I17" s="3" t="s">
         <v>123</v>
@@ -3781,7 +3515,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="30.75">
+    <row r="18" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="36">
         <v>17</v>
       </c>
@@ -3803,12 +3537,12 @@
         <v>14</v>
       </c>
       <c r="H18" s="40" t="s">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="I18" s="40"/>
       <c r="J18" s="40"/>
     </row>
-    <row r="19" spans="1:10" ht="32.25">
+    <row r="19" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A19" s="11">
         <v>18</v>
       </c>
@@ -3835,7 +3569,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="18.75">
+    <row r="22" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
       <c r="E22" s="34" t="s">
         <v>128</v>
       </c>
@@ -3846,25 +3580,25 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="H2:H19">
-    <cfRule type="containsText" dxfId="60" priority="1" operator="containsText" text="Overdue">
+    <cfRule type="containsText" dxfId="6" priority="1" operator="containsText" text="Overdue">
       <formula>NOT(ISERROR(SEARCH("Overdue",H2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="59" priority="2" operator="containsText" text="Blocked">
+    <cfRule type="containsText" dxfId="5" priority="2" operator="containsText" text="Blocked">
       <formula>NOT(ISERROR(SEARCH("Blocked",H2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="58" priority="3" operator="containsText" text="Cancelled">
+    <cfRule type="containsText" dxfId="4" priority="3" operator="containsText" text="Cancelled">
       <formula>NOT(ISERROR(SEARCH("Cancelled",H2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="57" priority="4" operator="containsText" text="Completed">
+    <cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="Completed">
       <formula>NOT(ISERROR(SEARCH("Completed",H2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="56" priority="5" operator="containsText" text="In Progress">
+    <cfRule type="containsText" dxfId="2" priority="5" operator="containsText" text="In Progress">
       <formula>NOT(ISERROR(SEARCH("In Progress",H2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="55" priority="6" operator="containsText" text="Planned">
+    <cfRule type="containsText" dxfId="1" priority="6" operator="containsText" text="Planned">
       <formula>NOT(ISERROR(SEARCH("Planned",H2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="54" priority="7" operator="containsText" text="Backlog">
+    <cfRule type="containsText" dxfId="0" priority="7" operator="containsText" text="Backlog">
       <formula>NOT(ISERROR(SEARCH("Backlog",H2)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3886,14 +3620,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23" style="3" customWidth="1"/>
     <col min="2" max="2" width="28.85546875" style="3" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32.5703125" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>129</v>
       </c>
@@ -3904,7 +3638,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="30">
+    <row r="2" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>89</v>
       </c>
@@ -3915,7 +3649,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="30">
+    <row r="3" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>96</v>
       </c>
@@ -3926,7 +3660,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="30">
+    <row r="4" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>110</v>
       </c>
@@ -3937,11 +3671,11 @@
         <v>136</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>129</v>
       </c>
@@ -3952,7 +3686,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>89</v>
       </c>
@@ -3963,7 +3697,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>89</v>
       </c>
@@ -3974,7 +3708,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>96</v>
       </c>
@@ -3985,7 +3719,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>96</v>
       </c>
@@ -3996,7 +3730,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="1:3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>110</v>
       </c>
@@ -4007,7 +3741,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>110</v>
       </c>
@@ -4031,7 +3765,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9663B98E-C5B6-4548-8DAD-F2D424BDE9B8}">
   <dimension ref="A1:J36"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.85546875" customWidth="1"/>
     <col min="2" max="2" width="18.5703125" customWidth="1"/>
@@ -4043,19 +3777,19 @@
     <col min="10" max="10" width="50.7109375" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="18.75">
-      <c r="A1" s="50" t="s">
+    <row r="1" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="51" t="s">
         <v>144</v>
       </c>
-      <c r="B1" s="50"/>
-      <c r="C1" s="50"/>
-    </row>
-    <row r="2" spans="1:10" ht="18.75">
+      <c r="B1" s="51"/>
+      <c r="C1" s="51"/>
+    </row>
+    <row r="2" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A2" s="6"/>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
     </row>
-    <row r="3" spans="1:10" ht="18.75">
+    <row r="3" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>145</v>
       </c>
@@ -4065,7 +3799,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>147</v>
       </c>
@@ -4091,7 +3825,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="30">
+    <row r="6" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>1</v>
       </c>
@@ -4117,7 +3851,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="30">
+    <row r="7" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>2</v>
       </c>
@@ -4143,7 +3877,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="30">
+    <row r="8" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>3</v>
       </c>
@@ -4169,7 +3903,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="30">
+    <row r="9" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>4</v>
       </c>
@@ -4195,7 +3929,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="30">
+    <row r="10" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>5</v>
       </c>
@@ -4221,7 +3955,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="30">
+    <row r="11" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>6</v>
       </c>
@@ -4247,7 +3981,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="30">
+    <row r="12" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>7</v>
       </c>
@@ -4273,7 +4007,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="30">
+    <row r="13" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>8</v>
       </c>
@@ -4299,7 +4033,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="30">
+    <row r="14" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>9</v>
       </c>
@@ -4325,7 +4059,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="30">
+    <row r="15" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>10</v>
       </c>
@@ -4351,7 +4085,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="30">
+    <row r="16" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>11</v>
       </c>
@@ -4377,7 +4111,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="30">
+    <row r="17" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>12</v>
       </c>
@@ -4403,7 +4137,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="30">
+    <row r="18" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>13</v>
       </c>
@@ -4429,7 +4163,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="30">
+    <row r="19" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>14</v>
       </c>
@@ -4455,7 +4189,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="30">
+    <row r="20" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>15</v>
       </c>
@@ -4481,7 +4215,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="30">
+    <row r="21" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>16</v>
       </c>
@@ -4507,7 +4241,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="30">
+    <row r="22" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>17</v>
       </c>
@@ -4533,7 +4267,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="30">
+    <row r="23" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>18</v>
       </c>
@@ -4559,7 +4293,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="30">
+    <row r="24" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>19</v>
       </c>
@@ -4585,7 +4319,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="30">
+    <row r="25" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>20</v>
       </c>
@@ -4611,7 +4345,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="30">
+    <row r="26" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>21</v>
       </c>
@@ -4637,7 +4371,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="30">
+    <row r="27" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>22</v>
       </c>
@@ -4663,7 +4397,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ht="30">
+    <row r="28" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>23</v>
       </c>
@@ -4689,7 +4423,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="30">
+    <row r="29" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>24</v>
       </c>
@@ -4715,7 +4449,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="30">
+    <row r="30" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>25</v>
       </c>
@@ -4741,7 +4475,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="30">
+    <row r="31" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
         <v>26</v>
       </c>
@@ -4767,7 +4501,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="30">
+    <row r="32" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <v>27</v>
       </c>
@@ -4793,7 +4527,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="33" spans="1:10" ht="30">
+    <row r="33" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <v>28</v>
       </c>
@@ -4819,7 +4553,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="34" spans="1:10" ht="30">
+    <row r="34" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>29</v>
       </c>
@@ -4845,7 +4579,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="35" spans="1:10" ht="30">
+    <row r="35" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <v>30</v>
       </c>
@@ -4871,7 +4605,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="36" spans="1:10" ht="30.75">
+    <row r="36" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
         <v>31</v>
       </c>
@@ -4909,65 +4643,65 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90B00C9A-DBF0-4699-96A2-B1424F93F245}">
   <dimension ref="A1:A12"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="68" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="24.75">
+    <row r="2" spans="1:1" ht="24.75" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="17.25">
+    <row r="3" spans="1:1" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="17.25">
+    <row r="4" spans="1:1" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="17.25">
+    <row r="5" spans="1:1" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="17.25">
+    <row r="6" spans="1:1" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="7" spans="1:1" ht="17.25">
+    <row r="7" spans="1:1" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A7" s="46" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="8" spans="1:1" ht="17.25">
+    <row r="8" spans="1:1" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="9" spans="1:1" ht="17.25">
+    <row r="9" spans="1:1" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A9" s="14"/>
     </row>
-    <row r="10" spans="1:1">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>228</v>
       </c>
     </row>
-    <row r="11" spans="1:1">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="12" spans="1:1">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>230</v>
       </c>
@@ -4983,7 +4717,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:I27"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="17" customWidth="1"/>
@@ -4996,7 +4730,7 @@
     <col min="9" max="9" width="24.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>231</v>
       </c>
@@ -5022,7 +4756,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>238</v>
       </c>
@@ -5040,7 +4774,7 @@
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>242</v>
       </c>
@@ -5058,7 +4792,7 @@
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>245</v>
       </c>
@@ -5076,7 +4810,7 @@
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
     </row>
-    <row r="5" spans="1:8">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>247</v>
       </c>
@@ -5094,7 +4828,7 @@
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
     </row>
-    <row r="6" spans="1:8">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>250</v>
       </c>
@@ -5112,7 +4846,7 @@
       <c r="G6" s="3"/>
       <c r="H6" s="3"/>
     </row>
-    <row r="7" spans="1:8">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>253</v>
       </c>
@@ -5130,7 +4864,7 @@
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
     </row>
-    <row r="8" spans="1:8">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>257</v>
       </c>
@@ -5148,7 +4882,7 @@
       <c r="G8" s="3"/>
       <c r="H8" s="3"/>
     </row>
-    <row r="9" spans="1:8">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>260</v>
       </c>
@@ -5166,7 +4900,7 @@
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
     </row>
-    <row r="10" spans="1:8">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>262</v>
       </c>
@@ -5184,7 +4918,7 @@
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
     </row>
-    <row r="11" spans="1:8">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>264</v>
       </c>
@@ -5202,17 +4936,17 @@
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
     </row>
-    <row r="13" spans="1:8">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="16" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="17.25">
+    <row r="14" spans="1:8" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A14" s="15" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="15" spans="1:8">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>238</v>
       </c>
@@ -5229,7 +4963,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="30">
+    <row r="16" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>267</v>
       </c>
@@ -5246,7 +4980,7 @@
         <v>6.2</v>
       </c>
     </row>
-    <row r="17" spans="1:9">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>271</v>
       </c>
@@ -5263,7 +4997,7 @@
         <v>3.8</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="30">
+    <row r="18" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>275</v>
       </c>
@@ -5280,12 +5014,12 @@
         <v>5.0999999999999996</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="17.25">
+    <row r="21" spans="1:9" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A21" s="15" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="76.5">
+    <row r="22" spans="1:9" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A22" s="20" t="s">
         <v>280</v>
       </c>
@@ -5314,7 +5048,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="23" spans="1:9">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>238</v>
       </c>
@@ -5343,7 +5077,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="24" spans="1:9">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>267</v>
       </c>
@@ -5372,7 +5106,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:9">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>271</v>
       </c>
@@ -5401,7 +5135,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:9">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>275</v>
       </c>
@@ -5430,7 +5164,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:9">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>289</v>
       </c>
@@ -5475,38 +5209,38 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECC2616A-C033-438B-B356-AD1E491AEBF1}">
   <dimension ref="A1:A6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>291</v>
       </c>
     </row>
-    <row r="3" spans="1:1">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>292</v>
       </c>
     </row>
-    <row r="4" spans="1:1">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>293</v>
       </c>
     </row>
-    <row r="5" spans="1:1">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="6" spans="1:1">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>295</v>
       </c>
@@ -5522,14 +5256,14 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9BEC3059-1ED5-48E0-970B-2136BB7F4A2A}">
   <dimension ref="A1:A43"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
         <v>296</v>
       </c>
     </row>
-    <row r="43" spans="1:1">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" s="16" t="s">
         <v>297</v>
       </c>

</xml_diff>